<commit_message>
Update code and documentation
</commit_message>
<xml_diff>
--- a/2026-DeployableBridges/DCR curve.xlsx
+++ b/2026-DeployableBridges/DCR curve.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\My Drive\Dr. Zhu\Code\Sim-FAST\2026-DeployableBridges\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{13BBF0A4-2D57-48CB-B18F-8C06BA0464A0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4AF02140-2EFE-471B-9499-4705B8E6AB78}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="510" yWindow="360" windowWidth="27885" windowHeight="20400" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="13900" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -2289,37 +2289,37 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="11"/>
                 <c:pt idx="0">
-                  <c:v>0.1196</c:v>
+                  <c:v>0.3926</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>0.1177</c:v>
+                  <c:v>0.38640000000000002</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>0.1158</c:v>
+                  <c:v>0.38</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>0.1137</c:v>
+                  <c:v>0.37330000000000002</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>0.1115</c:v>
+                  <c:v>0.36630000000000001</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>0.10929999999999999</c:v>
+                  <c:v>0.35909999999999997</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>0.107</c:v>
+                  <c:v>0.35160000000000002</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>0.1046</c:v>
+                  <c:v>0.34389999999999998</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>0.1021</c:v>
+                  <c:v>0.33589999999999998</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>9.1300000000000006E-2</c:v>
+                  <c:v>0.3105</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>4.99E-2</c:v>
+                  <c:v>0.20849999999999999</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -3699,7 +3699,7 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
-                  <c:v>0.1196</c:v>
+                  <c:v>0.3926</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -7823,10 +7823,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="B2:V14"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="B2:X14"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
-    <row r="2" spans="2:22" x14ac:dyDescent="0.25">
+    <row r="2" spans="2:24" x14ac:dyDescent="0.35">
       <c r="B2" t="s">
         <v>2</v>
       </c>
@@ -7846,7 +7846,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="3" spans="2:22" x14ac:dyDescent="0.25">
+    <row r="3" spans="2:24" x14ac:dyDescent="0.35">
       <c r="B3" t="s">
         <v>1</v>
       </c>
@@ -7893,7 +7893,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="4" spans="2:22" x14ac:dyDescent="0.25">
+    <row r="4" spans="2:24" x14ac:dyDescent="0.35">
       <c r="B4">
         <v>0</v>
       </c>
@@ -7916,7 +7916,7 @@
         <v>0</v>
       </c>
       <c r="L4">
-        <v>0.1196</v>
+        <v>0.3926</v>
       </c>
       <c r="N4">
         <v>0</v>
@@ -7934,13 +7934,13 @@
         <v>0.14169999999999999</v>
       </c>
       <c r="U4">
-        <v>0.1196</v>
+        <v>0.3926</v>
       </c>
       <c r="V4">
         <v>0.30570000000000003</v>
       </c>
     </row>
-    <row r="5" spans="2:22" x14ac:dyDescent="0.25">
+    <row r="5" spans="2:24" x14ac:dyDescent="0.35">
       <c r="B5">
         <v>0.1</v>
       </c>
@@ -7963,7 +7963,7 @@
         <v>0.1</v>
       </c>
       <c r="L5">
-        <v>0.1177</v>
+        <v>0.38640000000000002</v>
       </c>
       <c r="N5">
         <v>0.1</v>
@@ -7972,7 +7972,7 @@
         <v>0.2954</v>
       </c>
     </row>
-    <row r="6" spans="2:22" x14ac:dyDescent="0.25">
+    <row r="6" spans="2:24" x14ac:dyDescent="0.35">
       <c r="B6">
         <v>0.2</v>
       </c>
@@ -7995,7 +7995,7 @@
         <v>0.2</v>
       </c>
       <c r="L6">
-        <v>0.1158</v>
+        <v>0.38</v>
       </c>
       <c r="N6">
         <v>0.2</v>
@@ -8004,7 +8004,7 @@
         <v>0.27879999999999999</v>
       </c>
     </row>
-    <row r="7" spans="2:22" x14ac:dyDescent="0.25">
+    <row r="7" spans="2:24" x14ac:dyDescent="0.35">
       <c r="B7">
         <v>0.3</v>
       </c>
@@ -8027,7 +8027,7 @@
         <v>0.3</v>
       </c>
       <c r="L7">
-        <v>0.1137</v>
+        <v>0.37330000000000002</v>
       </c>
       <c r="N7">
         <v>0.3</v>
@@ -8036,7 +8036,7 @@
         <v>0.2591</v>
       </c>
     </row>
-    <row r="8" spans="2:22" x14ac:dyDescent="0.25">
+    <row r="8" spans="2:24" x14ac:dyDescent="0.35">
       <c r="B8">
         <v>0.4</v>
       </c>
@@ -8059,7 +8059,7 @@
         <v>0.4</v>
       </c>
       <c r="L8">
-        <v>0.1115</v>
+        <v>0.36630000000000001</v>
       </c>
       <c r="N8">
         <v>0.4</v>
@@ -8068,7 +8068,7 @@
         <v>0.24610000000000001</v>
       </c>
     </row>
-    <row r="9" spans="2:22" x14ac:dyDescent="0.25">
+    <row r="9" spans="2:24" x14ac:dyDescent="0.35">
       <c r="B9">
         <v>0.5</v>
       </c>
@@ -8091,7 +8091,7 @@
         <v>0.5</v>
       </c>
       <c r="L9">
-        <v>0.10929999999999999</v>
+        <v>0.35909999999999997</v>
       </c>
       <c r="N9">
         <v>0.5</v>
@@ -8100,7 +8100,7 @@
         <v>0.23469999999999999</v>
       </c>
     </row>
-    <row r="10" spans="2:22" x14ac:dyDescent="0.25">
+    <row r="10" spans="2:24" x14ac:dyDescent="0.35">
       <c r="B10">
         <v>0.6</v>
       </c>
@@ -8123,7 +8123,7 @@
         <v>0.6</v>
       </c>
       <c r="L10">
-        <v>0.107</v>
+        <v>0.35160000000000002</v>
       </c>
       <c r="N10">
         <v>0.6</v>
@@ -8132,7 +8132,7 @@
         <v>0.22209999999999999</v>
       </c>
     </row>
-    <row r="11" spans="2:22" x14ac:dyDescent="0.25">
+    <row r="11" spans="2:24" x14ac:dyDescent="0.35">
       <c r="B11">
         <v>0.7</v>
       </c>
@@ -8155,7 +8155,7 @@
         <v>0.7</v>
       </c>
       <c r="L11">
-        <v>0.1046</v>
+        <v>0.34389999999999998</v>
       </c>
       <c r="N11">
         <v>0.7</v>
@@ -8164,7 +8164,7 @@
         <v>0.20830000000000001</v>
       </c>
     </row>
-    <row r="12" spans="2:22" x14ac:dyDescent="0.25">
+    <row r="12" spans="2:24" x14ac:dyDescent="0.35">
       <c r="B12">
         <v>0.8</v>
       </c>
@@ -8187,7 +8187,7 @@
         <v>0.8</v>
       </c>
       <c r="L12">
-        <v>0.1021</v>
+        <v>0.33589999999999998</v>
       </c>
       <c r="N12">
         <v>0.8</v>
@@ -8196,7 +8196,7 @@
         <v>0.19259999999999999</v>
       </c>
     </row>
-    <row r="13" spans="2:22" x14ac:dyDescent="0.25">
+    <row r="13" spans="2:24" x14ac:dyDescent="0.35">
       <c r="B13">
         <v>0.9</v>
       </c>
@@ -8219,7 +8219,7 @@
         <v>0.9</v>
       </c>
       <c r="L13">
-        <v>9.1300000000000006E-2</v>
+        <v>0.3105</v>
       </c>
       <c r="N13">
         <v>0.9</v>
@@ -8228,7 +8228,7 @@
         <v>0.17349999999999999</v>
       </c>
     </row>
-    <row r="14" spans="2:22" x14ac:dyDescent="0.25">
+    <row r="14" spans="2:24" x14ac:dyDescent="0.35">
       <c r="B14">
         <v>1</v>
       </c>
@@ -8251,13 +8251,16 @@
         <v>1</v>
       </c>
       <c r="L14">
-        <v>4.99E-2</v>
+        <v>0.20849999999999999</v>
       </c>
       <c r="N14">
         <v>1</v>
       </c>
       <c r="O14">
         <v>0.13830000000000001</v>
+      </c>
+      <c r="X14">
+        <v>0.28570000000000001</v>
       </c>
     </row>
   </sheetData>

</xml_diff>